<commit_message>
chore: update stufe-5/labor/migration-test-ig-ptdata-1968 pages
</commit_message>
<xml_diff>
--- a/stufe-5/labor/migration-test-ig-ptdata-1968/observations-summary.xlsx
+++ b/stufe-5/labor/migration-test-ig-ptdata-1968/observations-summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="35">
   <si>
     <t>Profile</t>
   </si>
@@ -47,55 +47,76 @@
     <t>Method</t>
   </si>
   <si>
-    <t>ISiKAlkoholAbusus</t>
-  </si>
-  <si>
-    <t>ISiK Alkohol Abusus</t>
-  </si>
-  <si>
-    <t>Observation Category Codes#social-history</t>
+    <t>ISiKLaboruntersuchung</t>
+  </si>
+  <si>
+    <t>null#laboratory</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>null#15167005, null#74043-1</t>
+    <t>null#null</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/observation-codes|4.0.1 (example)</t>
   </si>
   <si>
-    <t>dateTimeĵ, Periodĵ</t>
-  </si>
-  <si>
-    <t>CodeableConceptĵ</t>
+    <t>dateTimeĵ, Periodĵ, Timingĵ, instantĵ</t>
+  </si>
+  <si>
+    <t>Quantityĵ, CodeableConceptĵ, stringĵ, booleanĵ, integerĵ, Rangeĵ, Ratioĵ, SampledDataĵ, timeĵ, dateTimeĵ, Periodĵ</t>
   </si>
   <si>
     <t>optional</t>
   </si>
   <si>
-    <t>ISiKRaucherStatus</t>
-  </si>
-  <si>
-    <t>ISiK Raucherstatus</t>
-  </si>
-  <si>
-    <t>null#77176002, null#72166-2</t>
-  </si>
-  <si>
-    <t>ISiKSchwangerschaftsstatus</t>
-  </si>
-  <si>
-    <t>ISiK Schwangerschaftsstatus</t>
-  </si>
-  <si>
-    <t>LOINC#82810-3</t>
-  </si>
-  <si>
-    <t>ISiKStillstatus</t>
-  </si>
-  <si>
-    <t>null#413712001, null#63895-7</t>
+    <t>ISiKLaboruntersuchungCRP</t>
+  </si>
+  <si>
+    <t>null#null, null#55235003</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungGFR</t>
+  </si>
+  <si>
+    <t>null#null, null#80274001</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungHb</t>
+  </si>
+  <si>
+    <t>null#null, null#416125006</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungPCT</t>
+  </si>
+  <si>
+    <t>null#null, null#418752001</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungSerumkreatinin</t>
+  </si>
+  <si>
+    <t>null#null, null#70901006</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungThrombozyten</t>
+  </si>
+  <si>
+    <t>null#null, null#365632008</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungTroponin</t>
+  </si>
+  <si>
+    <t>null#null, null#105000003</t>
+  </si>
+  <si>
+    <t>ISiKLaboruntersuchungTSH</t>
+  </si>
+  <si>
+    <t>null#null, null#61167004</t>
   </si>
 </sst>
 </file>
@@ -229,7 +250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -272,139 +293,314 @@
         <v>11</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="E2" t="s" s="2">
-        <v>15</v>
-      </c>
       <c r="F2" t="s" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B3" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s" s="2">
-        <v>22</v>
-      </c>
       <c r="F3" t="s" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3" t="s" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H3" t="s" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I3" t="s" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J3" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K3" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G4" t="s" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H4" t="s" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4" t="s" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K4" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K5" t="s" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="2">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="B5" t="s" s="2">
-        <v>26</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s" s="2">
+      <c r="F6" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H6" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I6" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K6" t="s" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="F5" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="G5" t="s" s="2">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="I5" t="s" s="2">
-        <v>19</v>
-      </c>
-      <c r="J5" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="K5" t="s" s="2">
-        <v>14</v>
+      <c r="B7" t="s" s="2">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="F7" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H7" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I7" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J7" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J8" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I9" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J9" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G10" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H10" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I10" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J10" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="K10" t="s" s="2">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>